<commit_message>
FD correlation with richness exploration FD differences between germ and adult plant traits Ms 0 updated with description of preliminar results
</commit_message>
<xml_diff>
--- a/results/summary community level analysis.xlsx
+++ b/results/summary community level analysis.xlsx
@@ -438,34 +438,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
@@ -477,43 +453,67 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -522,19 +522,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3236,6 +3236,106 @@
       <xdr:spPr>
         <a:xfrm flipV="1">
           <a:off x="5905500" y="6477000"/>
+          <a:ext cx="609600" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="92D050"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>27216</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>27216</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>646341</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>179616</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="56" name="Conector recto de flecha 55"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1877787" y="6640287"/>
+          <a:ext cx="619125" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>102057</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>6807</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="57" name="Conector recto de flecha 56"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="5871482" y="537486"/>
           <a:ext cx="609600" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -3537,9 +3637,9 @@
     <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="10" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="10" style="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" style="1" customWidth="1"/>
     <col min="10" max="12" width="10" style="1" customWidth="1"/>
     <col min="13" max="13" width="4.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="10" style="1" customWidth="1"/>
@@ -3551,16 +3651,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="6"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="17"/>
       <c r="G1" s="35" t="s">
         <v>28</v>
       </c>
@@ -3568,12 +3668,12 @@
       <c r="I1" s="36"/>
       <c r="J1" s="36"/>
       <c r="K1" s="37"/>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="6"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="17"/>
       <c r="P1" s="35" t="s">
         <v>27</v>
       </c>
@@ -3583,529 +3683,529 @@
       <c r="T1" s="37"/>
     </row>
     <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="3" t="s">
+      <c r="P2" s="4"/>
+      <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="4" t="s">
+      <c r="C3" s="18"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18" t="s">
+      <c r="I3" s="15"/>
+      <c r="J3" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="17"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18" t="s">
+      <c r="L3" s="18"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="34" t="s">
+      <c r="O3" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="18"/>
-      <c r="T3" s="19" t="s">
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="21"/>
-      <c r="T4" s="22"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="10"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="20" t="s">
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="32" t="s">
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="22"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="10"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="7" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="7" t="s">
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="21" t="s">
+      <c r="Q6" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="22"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="10"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="2" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="20" t="s">
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="32" t="s">
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="22"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="10"/>
     </row>
     <row r="8" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
-      <c r="O8" s="33"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="24"/>
-      <c r="R8" s="24"/>
-      <c r="S8" s="24"/>
-      <c r="T8" s="25"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="13"/>
+      <c r="S8" s="13"/>
+      <c r="T8" s="11"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18" t="s">
+      <c r="D9" s="15"/>
+      <c r="E9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="14"/>
+      <c r="G9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="31" t="s">
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="19" t="s">
+      <c r="O9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="P9" s="4" t="s">
+      <c r="P9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q9" s="18" t="s">
+      <c r="Q9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="R9" s="18"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="19" t="s">
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="14" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="21"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="12"/>
       <c r="N10" s="28"/>
-      <c r="O10" s="22"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21"/>
-      <c r="T10" s="22"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="10"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="2" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="22" t="s">
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="21"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="12"/>
       <c r="N11" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="O11" s="22" t="s">
+      <c r="O11" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
-      <c r="T11" s="22"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="10"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="21"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="12"/>
       <c r="N12" s="28"/>
-      <c r="O12" s="22"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="21"/>
-      <c r="S12" s="21"/>
-      <c r="T12" s="22"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="10"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="2" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="21"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="12"/>
       <c r="N13" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="O13" s="22"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="21"/>
-      <c r="S13" s="21"/>
-      <c r="T13" s="22"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="10"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="7" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="21" t="s">
+      <c r="H14" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="21"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="12"/>
       <c r="N14" s="28"/>
-      <c r="O14" s="22"/>
-      <c r="P14" s="7" t="s">
+      <c r="O14" s="10"/>
+      <c r="P14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="21"/>
-      <c r="S14" s="21" t="s">
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="T14" s="22" t="s">
+      <c r="T14" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="2" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
-      <c r="S15" s="21"/>
-      <c r="T15" s="22"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="10"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="21"/>
-      <c r="S16" s="21"/>
-      <c r="T16" s="22"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="10"/>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="2" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="20"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="21"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="27" t="s">
+      <c r="E17" s="12"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="21"/>
-      <c r="S17" s="21"/>
-      <c r="T17" s="22"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="10"/>
     </row>
     <row r="18" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="23"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="29"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="24"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="25"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="24"/>
-      <c r="R18" s="24"/>
-      <c r="S18" s="24"/>
-      <c r="T18" s="25"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="11"/>
     </row>
     <row r="20" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="1:20" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="16"/>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="33"/>
+      <c r="C21" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="6"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="17"/>
       <c r="G21" s="35" t="s">
         <v>28</v>
       </c>
@@ -4113,515 +4213,514 @@
       <c r="I21" s="36"/>
       <c r="J21" s="36"/>
       <c r="K21" s="37"/>
-      <c r="L21" s="4" t="s">
+      <c r="L21" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="5" t="s">
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
-      <c r="T21" s="6"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="17"/>
     </row>
     <row r="22" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="12"/>
-      <c r="H22" s="3" t="s">
+      <c r="G22" s="4"/>
+      <c r="H22" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K22" s="13" t="s">
+      <c r="K22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L22" s="12" t="s">
+      <c r="L22" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M22" s="3" t="s">
+      <c r="M22" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="N22" s="3" t="s">
+      <c r="N22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O22" s="13" t="s">
+      <c r="O22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="P22" s="12"/>
-      <c r="Q22" s="3" t="s">
+      <c r="P22" s="4"/>
+      <c r="Q22" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="R22" s="3" t="s">
+      <c r="R22" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S22" s="3" t="s">
+      <c r="S22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="T22" s="13" t="s">
+      <c r="T22" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="31" t="s">
+      <c r="C23" s="18"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="4" t="s">
+      <c r="F23" s="14"/>
+      <c r="G23" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I23" s="18"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="31" t="s">
+      <c r="I23" s="15"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="O23" s="19"/>
-      <c r="P23" s="4" t="s">
+      <c r="O23" s="14"/>
+      <c r="P23" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="31" t="s">
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="T23" s="19"/>
+      <c r="T23" s="14"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="12"/>
       <c r="E24" s="28"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
       <c r="J24" s="28"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="20"/>
-      <c r="M24" s="21"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="12"/>
       <c r="N24" s="28"/>
-      <c r="O24" s="22"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="21"/>
-      <c r="R24" s="21"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
       <c r="S24" s="28"/>
-      <c r="T24" s="22"/>
+      <c r="T24" s="10"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="2" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
       <c r="J25" s="28"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="20"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="21"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="7"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="21"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
       <c r="S25" s="28"/>
-      <c r="T25" s="22"/>
+      <c r="T25" s="10"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="7" t="s">
+      <c r="A26" s="8"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="I26" s="21"/>
+      <c r="I26" s="12"/>
       <c r="J26" s="28"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="20"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="21"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="7" t="s">
+      <c r="K26" s="10"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="21"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
       <c r="S26" s="28"/>
-      <c r="T26" s="22"/>
+      <c r="T26" s="10"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="2" t="s">
+      <c r="A27" s="8"/>
+      <c r="B27" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="21"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
       <c r="J27" s="28"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="20"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="21"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="21"/>
-      <c r="R27" s="21"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="12"/>
+      <c r="R27" s="12"/>
       <c r="S27" s="28"/>
-      <c r="T27" s="22"/>
+      <c r="T27" s="10"/>
     </row>
     <row r="28" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
       <c r="J28" s="29"/>
-      <c r="K28" s="25"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="24"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="25"/>
-      <c r="P28" s="8"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="24"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="9"/>
+      <c r="Q28" s="13"/>
+      <c r="R28" s="13"/>
       <c r="S28" s="29"/>
-      <c r="T28" s="25"/>
+      <c r="T28" s="11"/>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="4" t="s">
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18" t="s">
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="K29" s="19"/>
-      <c r="L29" s="17" t="s">
+      <c r="K29" s="14"/>
+      <c r="L29" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="19"/>
-      <c r="P29" s="4" t="s">
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="14"/>
+      <c r="P29" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q29" s="18"/>
-      <c r="R29" s="18"/>
-      <c r="S29" s="18" t="s">
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="T29" s="19"/>
+      <c r="T29" s="14"/>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="20"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="22"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="21"/>
-      <c r="R30" s="21"/>
-      <c r="S30" s="21"/>
-      <c r="T30" s="22"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="12"/>
+      <c r="R30" s="12"/>
+      <c r="S30" s="12"/>
+      <c r="T30" s="10"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-      <c r="B31" s="2" t="s">
+      <c r="A31" s="8"/>
+      <c r="B31" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21" t="s">
+      <c r="C31" s="19"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="F31" s="22"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="20"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="21" t="s">
+      <c r="F31" s="10"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="O31" s="22"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="21"/>
-      <c r="R31" s="21"/>
-      <c r="S31" s="21"/>
-      <c r="T31" s="22"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="10"/>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="20"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="22"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="21"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="22"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="12"/>
+      <c r="R32" s="12"/>
+      <c r="S32" s="12"/>
+      <c r="T32" s="10"/>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="B33" s="2" t="s">
+      <c r="A33" s="8"/>
+      <c r="B33" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C33" s="20"/>
+      <c r="C33" s="19"/>
       <c r="D33" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="E33" s="21" t="s">
+      <c r="E33" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="F33" s="22"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="22"/>
-      <c r="L33" s="20"/>
-      <c r="M33" s="21"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="21"/>
-      <c r="R33" s="21"/>
-      <c r="S33" s="21"/>
-      <c r="T33" s="22"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="8"/>
+      <c r="Q33" s="12"/>
+      <c r="R33" s="12"/>
+      <c r="S33" s="12"/>
+      <c r="T33" s="10"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="19"/>
       <c r="D34" s="28"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="7" t="s">
+      <c r="E34" s="12"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H34" s="21"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21" t="s">
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K34" s="22"/>
-      <c r="L34" s="20"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="21"/>
-      <c r="O34" s="22"/>
-      <c r="P34" s="7" t="s">
+      <c r="K34" s="10"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="Q34" s="21"/>
-      <c r="R34" s="21"/>
-      <c r="S34" s="21" t="s">
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="T34" s="22"/>
+      <c r="T34" s="10"/>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="2" t="s">
+      <c r="A35" s="8"/>
+      <c r="B35" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21" t="s">
+      <c r="D35" s="12"/>
+      <c r="E35" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F35" s="22"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="20"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="21" t="s">
+      <c r="F35" s="10"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="O35" s="22"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="21"/>
-      <c r="R35" s="21"/>
-      <c r="S35" s="21"/>
-      <c r="T35" s="22"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12"/>
+      <c r="T35" s="10"/>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
-      <c r="K36" s="22"/>
-      <c r="L36" s="20"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="21"/>
-      <c r="O36" s="22"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="21"/>
-      <c r="R36" s="21"/>
-      <c r="S36" s="21"/>
-      <c r="T36" s="22"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="12"/>
+      <c r="R36" s="12"/>
+      <c r="S36" s="12"/>
+      <c r="T36" s="10"/>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="2" t="s">
+      <c r="A37" s="8"/>
+      <c r="B37" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C37" s="20" t="s">
+      <c r="C37" s="19" t="s">
         <v>26</v>
       </c>
       <c r="D37" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E37" s="21"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="21"/>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="22"/>
-      <c r="L37" s="20"/>
-      <c r="M37" s="21"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="12"/>
       <c r="N37" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="O37" s="22"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="21"/>
-      <c r="R37" s="21"/>
-      <c r="S37" s="21"/>
-      <c r="T37" s="22"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="12"/>
+      <c r="R37" s="12"/>
+      <c r="S37" s="12"/>
+      <c r="T37" s="10"/>
     </row>
     <row r="38" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="23"/>
+      <c r="A38" s="9"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="24"/>
       <c r="D38" s="29"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
-      <c r="J38" s="24"/>
-      <c r="K38" s="25"/>
-      <c r="L38" s="23"/>
-      <c r="M38" s="24"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="13"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="13"/>
+      <c r="K38" s="11"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="13"/>
       <c r="N38" s="29"/>
-      <c r="O38" s="25"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="24"/>
-      <c r="R38" s="24"/>
-      <c r="S38" s="24"/>
-      <c r="T38" s="25"/>
+      <c r="O38" s="11"/>
+      <c r="P38" s="9"/>
+      <c r="Q38" s="13"/>
+      <c r="R38" s="13"/>
+      <c r="S38" s="13"/>
+      <c r="T38" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="238">
-    <mergeCell ref="K34:K38"/>
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="G21:K21"/>
@@ -4645,14 +4744,6 @@
     <mergeCell ref="I6:I8"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="K6:K8"/>
-    <mergeCell ref="G9:G13"/>
-    <mergeCell ref="H9:H13"/>
-    <mergeCell ref="I9:I13"/>
-    <mergeCell ref="J9:J13"/>
-    <mergeCell ref="K9:K13"/>
-    <mergeCell ref="M37:M38"/>
-    <mergeCell ref="N37:N38"/>
-    <mergeCell ref="O37:O38"/>
     <mergeCell ref="G3:G5"/>
     <mergeCell ref="H3:H5"/>
     <mergeCell ref="I3:I5"/>
@@ -4662,8 +4753,12 @@
     <mergeCell ref="L35:L36"/>
     <mergeCell ref="M35:M36"/>
     <mergeCell ref="N35:N36"/>
-    <mergeCell ref="O35:O36"/>
-    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="K34:K38"/>
     <mergeCell ref="C37:C38"/>
     <mergeCell ref="D37:D38"/>
     <mergeCell ref="E37:E38"/>
@@ -4672,6 +4767,16 @@
     <mergeCell ref="P34:P38"/>
     <mergeCell ref="Q34:Q38"/>
     <mergeCell ref="R34:R38"/>
+    <mergeCell ref="G9:G13"/>
+    <mergeCell ref="H9:H13"/>
+    <mergeCell ref="I9:I13"/>
+    <mergeCell ref="J9:J13"/>
+    <mergeCell ref="K9:K13"/>
+    <mergeCell ref="M37:M38"/>
+    <mergeCell ref="N37:N38"/>
+    <mergeCell ref="O37:O38"/>
+    <mergeCell ref="O35:O36"/>
+    <mergeCell ref="O29:O30"/>
     <mergeCell ref="S34:S38"/>
     <mergeCell ref="T34:T38"/>
     <mergeCell ref="B35:B36"/>
@@ -4696,12 +4801,19 @@
     <mergeCell ref="D31:D32"/>
     <mergeCell ref="E31:E32"/>
     <mergeCell ref="F31:F32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="O29:O30"/>
+    <mergeCell ref="A29:A38"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="Q26:Q28"/>
+    <mergeCell ref="R26:R28"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="P26:P28"/>
     <mergeCell ref="P29:P33"/>
     <mergeCell ref="Q29:Q33"/>
     <mergeCell ref="R29:R33"/>
@@ -4712,15 +4824,7 @@
     <mergeCell ref="M27:M28"/>
     <mergeCell ref="N27:N28"/>
     <mergeCell ref="O27:O28"/>
-    <mergeCell ref="A29:A38"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="Q26:Q28"/>
-    <mergeCell ref="R26:R28"/>
+    <mergeCell ref="B37:B38"/>
     <mergeCell ref="S26:S28"/>
     <mergeCell ref="T26:T28"/>
     <mergeCell ref="B27:B28"/>
@@ -4745,10 +4849,6 @@
     <mergeCell ref="N23:N24"/>
     <mergeCell ref="O23:O24"/>
     <mergeCell ref="P23:P25"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="P26:P28"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C21:F21"/>
@@ -4773,8 +4873,6 @@
     <mergeCell ref="O9:O10"/>
     <mergeCell ref="N9:N10"/>
     <mergeCell ref="M9:M10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="F9:F10"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="C9:C10"/>
@@ -4789,6 +4887,8 @@
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C6"/>
     <mergeCell ref="D15:D16"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="B15:B16"/>
@@ -4809,26 +4909,10 @@
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="L1:O1"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
@@ -4845,6 +4929,17 @@
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="A9:A18"/>
+    <mergeCell ref="T6:T8"/>
+    <mergeCell ref="S6:S8"/>
+    <mergeCell ref="R6:R8"/>
     <mergeCell ref="Q6:Q8"/>
     <mergeCell ref="P6:P8"/>
     <mergeCell ref="T3:T5"/>
@@ -4852,13 +4947,18 @@
     <mergeCell ref="R3:R5"/>
     <mergeCell ref="Q3:Q5"/>
     <mergeCell ref="P3:P5"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="A9:A18"/>
-    <mergeCell ref="T6:T8"/>
-    <mergeCell ref="S6:S8"/>
-    <mergeCell ref="R6:R8"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
new combined effect sizes figure
</commit_message>
<xml_diff>
--- a/results/summary community level analysis.xlsx
+++ b/results/summary community level analysis.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="33">
   <si>
     <t>Trait group</t>
   </si>
@@ -465,100 +465,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
@@ -569,6 +482,93 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3968,56 +3968,6 @@
         <a:ln w="28575">
           <a:solidFill>
             <a:srgbClr val="92D050"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>20410</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>18317</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>188407</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="106" name="Conector recto de flecha 105"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18439379" y="2399567"/>
-          <a:ext cx="646340" cy="170090"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="28575">
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
           </a:solidFill>
           <a:tailEnd type="triangle"/>
         </a:ln>
@@ -4684,40 +4634,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="27" t="s">
+      <c r="B1" s="53"/>
+      <c r="C1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="27" t="s">
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="27" t="s">
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="27" t="s">
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="36"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="23"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
@@ -4790,98 +4740,98 @@
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="34"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="32" t="s">
+      <c r="C3" s="51"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28" t="s">
+      <c r="I3" s="35"/>
+      <c r="J3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="29"/>
-      <c r="L3" s="41" t="s">
+      <c r="K3" s="37"/>
+      <c r="L3" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="27" t="s">
+      <c r="M3" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28" t="s">
+      <c r="N3" s="35"/>
+      <c r="O3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="P3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="47" t="s">
+      <c r="Q3" s="35"/>
+      <c r="R3" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="S3" s="27" t="s">
+      <c r="S3" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="T3" s="28"/>
-      <c r="U3" s="28"/>
-      <c r="V3" s="28"/>
-      <c r="W3" s="28" t="s">
+      <c r="T3" s="35"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="35"/>
+      <c r="W3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="X3" s="47"/>
+      <c r="X3" s="33"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="21"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="48"/>
-      <c r="S4" s="21"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="48"/>
+      <c r="A4" s="34"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="32"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="31"/>
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
+      <c r="W4" s="31"/>
+      <c r="X4" s="32"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="40" t="s">
+      <c r="A5" s="34"/>
+      <c r="B5" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="30" t="s">
+      <c r="C5" s="45"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="25" t="s">
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="42"/>
+      <c r="L5" s="39"/>
       <c r="M5" s="11" t="s">
         <v>27</v>
       </c>
@@ -4898,26 +4848,24 @@
         <v>22</v>
       </c>
       <c r="V5" s="5"/>
-      <c r="W5" s="10" t="s">
-        <v>22</v>
-      </c>
+      <c r="W5" s="10"/>
       <c r="X5" s="14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" s="21"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="42"/>
+      <c r="A6" s="34"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="39"/>
       <c r="M6" s="11" t="s">
         <v>28</v>
       </c>
@@ -4938,28 +4886,28 @@
       <c r="X6" s="14"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
-      <c r="B7" s="40" t="s">
+      <c r="A7" s="34"/>
+      <c r="B7" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="25" t="s">
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="42"/>
-      <c r="H7" s="30" t="s">
+      <c r="G7" s="39"/>
+      <c r="H7" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="25" t="s">
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="42"/>
+      <c r="L7" s="39"/>
       <c r="M7" s="11" t="s">
         <v>29</v>
       </c>
@@ -4988,18 +4936,18 @@
       </c>
     </row>
     <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="44"/>
+      <c r="A8" s="50"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="42"/>
       <c r="M8" s="12"/>
       <c r="N8" s="6"/>
       <c r="O8" s="6"/>
@@ -5014,164 +4962,164 @@
       <c r="X8" s="15"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28" t="s">
+      <c r="D9" s="35"/>
+      <c r="E9" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="41" t="s">
+      <c r="F9" s="35"/>
+      <c r="G9" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="34"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="29" t="s">
+      <c r="H9" s="51"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="K9" s="28" t="s">
+      <c r="K9" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="49" t="s">
+      <c r="L9" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="51"/>
-      <c r="N9" s="45"/>
-      <c r="O9" s="45"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="47"/>
-      <c r="S9" s="51"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
-      <c r="V9" s="45"/>
-      <c r="W9" s="45"/>
-      <c r="X9" s="47"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="27"/>
+      <c r="R9" s="33"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="27"/>
+      <c r="U9" s="27"/>
+      <c r="V9" s="27"/>
+      <c r="W9" s="27"/>
+      <c r="X9" s="33"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="50"/>
-      <c r="M10" s="52"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46"/>
-      <c r="P10" s="46"/>
-      <c r="Q10" s="46"/>
-      <c r="R10" s="48"/>
-      <c r="S10" s="52"/>
-      <c r="T10" s="46"/>
-      <c r="U10" s="46"/>
-      <c r="V10" s="46"/>
-      <c r="W10" s="46"/>
-      <c r="X10" s="48"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="36"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="28"/>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="32"/>
+      <c r="S10" s="30"/>
+      <c r="T10" s="28"/>
+      <c r="U10" s="28"/>
+      <c r="V10" s="28"/>
+      <c r="W10" s="28"/>
+      <c r="X10" s="32"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="40" t="s">
+      <c r="A11" s="34"/>
+      <c r="B11" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="25" t="s">
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="K11" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="L11" s="42"/>
-      <c r="M11" s="21" t="s">
+      <c r="L11" s="39"/>
+      <c r="M11" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="N11" s="23" t="s">
+      <c r="N11" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="O11" s="23"/>
-      <c r="P11" s="23"/>
-      <c r="Q11" s="23"/>
-      <c r="R11" s="48" t="s">
+      <c r="O11" s="31"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="S11" s="21" t="s">
+      <c r="S11" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="T11" s="23" t="s">
+      <c r="T11" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="U11" s="23"/>
-      <c r="V11" s="23"/>
-      <c r="W11" s="25" t="s">
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="X11" s="48"/>
+      <c r="X11" s="32"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="23"/>
-      <c r="Q12" s="23"/>
-      <c r="R12" s="48"/>
-      <c r="S12" s="21"/>
-      <c r="T12" s="23"/>
-      <c r="U12" s="23"/>
-      <c r="V12" s="23"/>
-      <c r="W12" s="25"/>
-      <c r="X12" s="48"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="39"/>
+      <c r="M12" s="34"/>
+      <c r="N12" s="31"/>
+      <c r="O12" s="31"/>
+      <c r="P12" s="31"/>
+      <c r="Q12" s="31"/>
+      <c r="R12" s="32"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="31"/>
+      <c r="U12" s="31"/>
+      <c r="V12" s="31"/>
+      <c r="W12" s="36"/>
+      <c r="X12" s="32"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A13" s="21"/>
-      <c r="B13" s="40" t="s">
+      <c r="A13" s="34"/>
+      <c r="B13" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="25" t="s">
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="K13" s="23"/>
-      <c r="L13" s="42" t="s">
+      <c r="K13" s="31"/>
+      <c r="L13" s="39" t="s">
         <v>21</v>
       </c>
       <c r="M13" s="11" t="s">
@@ -5200,18 +5148,18 @@
       <c r="X13" s="14"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="42"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="39"/>
       <c r="M14" s="11" t="s">
         <v>12</v>
       </c>
@@ -5234,22 +5182,22 @@
       <c r="X14" s="14"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A15" s="21"/>
-      <c r="B15" s="40" t="s">
+      <c r="A15" s="34"/>
+      <c r="B15" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="30" t="s">
+      <c r="C15" s="49"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="42"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="39"/>
       <c r="M15" s="11" t="s">
         <v>13</v>
       </c>
@@ -5274,18 +5222,18 @@
       <c r="X15" s="14"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A16" s="21"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="42"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="39"/>
       <c r="M16" s="11" t="s">
         <v>14</v>
       </c>
@@ -5312,26 +5260,26 @@
       <c r="X16" s="14"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A17" s="21"/>
-      <c r="B17" s="40" t="s">
+      <c r="A17" s="34"/>
+      <c r="B17" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="25" t="s">
+      <c r="C17" s="45"/>
+      <c r="D17" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="33" t="s">
+      <c r="F17" s="31"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="42"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="39"/>
       <c r="M17" s="11" t="s">
         <v>15</v>
       </c>
@@ -5354,18 +5302,18 @@
       <c r="X17" s="14"/>
     </row>
     <row r="18" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
-      <c r="L18" s="44"/>
+      <c r="A18" s="50"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="43"/>
+      <c r="K18" s="43"/>
+      <c r="L18" s="42"/>
       <c r="M18" s="12"/>
       <c r="N18" s="6"/>
       <c r="O18" s="6"/>
@@ -5381,40 +5329,40 @@
     </row>
     <row r="20" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="1:24" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="39"/>
-      <c r="C21" s="53" t="s">
+      <c r="B21" s="53"/>
+      <c r="C21" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="53" t="s">
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
-      <c r="K21" s="54"/>
-      <c r="L21" s="55"/>
-      <c r="M21" s="53" t="s">
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="N21" s="54"/>
-      <c r="O21" s="54"/>
-      <c r="P21" s="54"/>
-      <c r="Q21" s="54"/>
-      <c r="R21" s="55"/>
-      <c r="S21" s="53" t="s">
+      <c r="N21" s="25"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="25"/>
+      <c r="R21" s="26"/>
+      <c r="S21" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="T21" s="54"/>
-      <c r="U21" s="54"/>
-      <c r="V21" s="54"/>
-      <c r="W21" s="54"/>
-      <c r="X21" s="55"/>
+      <c r="T21" s="25"/>
+      <c r="U21" s="25"/>
+      <c r="V21" s="25"/>
+      <c r="W21" s="25"/>
+      <c r="X21" s="26"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
@@ -5487,88 +5435,88 @@
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="25" t="s">
+      <c r="C23" s="45"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="25" t="s">
+      <c r="F23" s="31"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="23"/>
-      <c r="L23" s="42"/>
-      <c r="M23" s="21" t="s">
+      <c r="K23" s="31"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="N23" s="23" t="s">
+      <c r="N23" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="O23" s="23"/>
-      <c r="P23" s="25"/>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="48"/>
-      <c r="S23" s="21" t="s">
+      <c r="O23" s="31"/>
+      <c r="P23" s="36"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="32"/>
+      <c r="S23" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="T23" s="23"/>
-      <c r="U23" s="23"/>
-      <c r="V23" s="25"/>
-      <c r="W23" s="23"/>
-      <c r="X23" s="48"/>
+      <c r="T23" s="31"/>
+      <c r="U23" s="31"/>
+      <c r="V23" s="36"/>
+      <c r="W23" s="31"/>
+      <c r="X23" s="32"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A24" s="21"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="42"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="23"/>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="23"/>
-      <c r="R24" s="48"/>
-      <c r="S24" s="21"/>
-      <c r="T24" s="23"/>
-      <c r="U24" s="23"/>
-      <c r="V24" s="25"/>
-      <c r="W24" s="23"/>
-      <c r="X24" s="48"/>
+      <c r="A24" s="34"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="39"/>
+      <c r="M24" s="34"/>
+      <c r="N24" s="31"/>
+      <c r="O24" s="31"/>
+      <c r="P24" s="36"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="34"/>
+      <c r="T24" s="31"/>
+      <c r="U24" s="31"/>
+      <c r="V24" s="36"/>
+      <c r="W24" s="31"/>
+      <c r="X24" s="32"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
-      <c r="B25" s="40" t="s">
+      <c r="A25" s="34"/>
+      <c r="B25" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="42"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="45"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="39"/>
       <c r="M25" s="11" t="s">
         <v>27</v>
       </c>
@@ -5589,18 +5537,18 @@
       <c r="X25" s="14"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A26" s="21"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="L26" s="42"/>
+      <c r="A26" s="34"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="39"/>
       <c r="M26" s="11" t="s">
         <v>28</v>
       </c>
@@ -5621,22 +5569,22 @@
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A27" s="21"/>
-      <c r="B27" s="40" t="s">
+      <c r="A27" s="34"/>
+      <c r="B27" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="42"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="42"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="39"/>
       <c r="M27" s="11" t="s">
         <v>29</v>
       </c>
@@ -5659,18 +5607,18 @@
       <c r="X27" s="14"/>
     </row>
     <row r="28" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22"/>
-      <c r="B28" s="43"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="44"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="43"/>
+      <c r="J28" s="43"/>
+      <c r="K28" s="43"/>
+      <c r="L28" s="42"/>
       <c r="M28" s="12"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
@@ -5685,152 +5633,152 @@
       <c r="X28" s="15"/>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="41"/>
-      <c r="H29" s="34" t="s">
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="41"/>
-      <c r="M29" s="51"/>
-      <c r="N29" s="45"/>
-      <c r="O29" s="45"/>
-      <c r="P29" s="45"/>
-      <c r="Q29" s="45"/>
-      <c r="R29" s="47"/>
-      <c r="S29" s="51"/>
-      <c r="T29" s="45"/>
-      <c r="U29" s="45"/>
-      <c r="V29" s="45"/>
-      <c r="W29" s="45"/>
-      <c r="X29" s="47"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="29"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="33"/>
+      <c r="S29" s="29"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
+      <c r="V29" s="27"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="33"/>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A30" s="21"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="23"/>
-      <c r="L30" s="42"/>
-      <c r="M30" s="52"/>
-      <c r="N30" s="46"/>
-      <c r="O30" s="46"/>
-      <c r="P30" s="46"/>
-      <c r="Q30" s="46"/>
-      <c r="R30" s="48"/>
-      <c r="S30" s="52"/>
-      <c r="T30" s="46"/>
-      <c r="U30" s="46"/>
-      <c r="V30" s="46"/>
-      <c r="W30" s="46"/>
-      <c r="X30" s="48"/>
+      <c r="A30" s="34"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="45"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="45"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="39"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="32"/>
+      <c r="S30" s="30"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
+      <c r="V30" s="28"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="32"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A31" s="21"/>
-      <c r="B31" s="40" t="s">
+      <c r="A31" s="34"/>
+      <c r="B31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23" t="s">
+      <c r="C31" s="45"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F31" s="23"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23" t="s">
+      <c r="F31" s="31"/>
+      <c r="G31" s="39"/>
+      <c r="H31" s="45"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="K31" s="23"/>
-      <c r="L31" s="42" t="s">
+      <c r="K31" s="31"/>
+      <c r="L31" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="M31" s="21" t="s">
+      <c r="M31" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23"/>
-      <c r="P31" s="23" t="s">
+      <c r="N31" s="31"/>
+      <c r="O31" s="31"/>
+      <c r="P31" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="Q31" s="23"/>
-      <c r="R31" s="48"/>
-      <c r="S31" s="21" t="s">
+      <c r="Q31" s="31"/>
+      <c r="R31" s="32"/>
+      <c r="S31" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="T31" s="23"/>
-      <c r="U31" s="23"/>
-      <c r="V31" s="23" t="s">
+      <c r="T31" s="31"/>
+      <c r="U31" s="31"/>
+      <c r="V31" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="W31" s="23"/>
-      <c r="X31" s="48" t="s">
+      <c r="W31" s="31"/>
+      <c r="X31" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A32" s="21"/>
-      <c r="B32" s="40"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="42"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="23"/>
-      <c r="R32" s="48"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="23"/>
-      <c r="U32" s="23"/>
-      <c r="V32" s="23"/>
-      <c r="W32" s="23"/>
-      <c r="X32" s="48"/>
+      <c r="A32" s="34"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="31"/>
+      <c r="J32" s="31"/>
+      <c r="K32" s="31"/>
+      <c r="L32" s="39"/>
+      <c r="M32" s="34"/>
+      <c r="N32" s="31"/>
+      <c r="O32" s="31"/>
+      <c r="P32" s="31"/>
+      <c r="Q32" s="31"/>
+      <c r="R32" s="32"/>
+      <c r="S32" s="34"/>
+      <c r="T32" s="31"/>
+      <c r="U32" s="31"/>
+      <c r="V32" s="31"/>
+      <c r="W32" s="31"/>
+      <c r="X32" s="32"/>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A33" s="21"/>
-      <c r="B33" s="40" t="s">
+      <c r="A33" s="34"/>
+      <c r="B33" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="C33" s="30"/>
-      <c r="D33" s="25" t="s">
+      <c r="C33" s="45"/>
+      <c r="D33" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
-      <c r="L33" s="42"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="45"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="39"/>
       <c r="M33" s="11" t="s">
         <v>30</v>
       </c>
@@ -5853,18 +5801,18 @@
       <c r="X33" s="14"/>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
-      <c r="B34" s="40"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="23"/>
-      <c r="L34" s="42"/>
+      <c r="A34" s="34"/>
+      <c r="B34" s="46"/>
+      <c r="C34" s="45"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="45"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="39"/>
       <c r="M34" s="11" t="s">
         <v>12</v>
       </c>
@@ -5887,28 +5835,28 @@
       <c r="X34" s="14"/>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A35" s="21"/>
-      <c r="B35" s="40" t="s">
+      <c r="A35" s="34"/>
+      <c r="B35" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="33" t="s">
+      <c r="C35" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23" t="s">
+      <c r="D35" s="31"/>
+      <c r="E35" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="F35" s="23"/>
-      <c r="G35" s="42" t="s">
+      <c r="F35" s="31"/>
+      <c r="G35" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="H35" s="30"/>
-      <c r="I35" s="23"/>
-      <c r="J35" s="23" t="s">
+      <c r="H35" s="45"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="K35" s="23"/>
-      <c r="L35" s="42" t="s">
+      <c r="K35" s="31"/>
+      <c r="L35" s="39" t="s">
         <v>22</v>
       </c>
       <c r="M35" s="11" t="s">
@@ -5935,18 +5883,18 @@
       <c r="X35" s="14"/>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A36" s="21"/>
-      <c r="B36" s="40"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="23"/>
-      <c r="L36" s="42"/>
+      <c r="A36" s="34"/>
+      <c r="B36" s="46"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="39"/>
       <c r="M36" s="11" t="s">
         <v>14</v>
       </c>
@@ -5973,24 +5921,24 @@
       </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A37" s="21"/>
-      <c r="B37" s="40" t="s">
+      <c r="A37" s="34"/>
+      <c r="B37" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="30"/>
-      <c r="D37" s="25" t="s">
+      <c r="C37" s="45"/>
+      <c r="D37" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="42"/>
-      <c r="H37" s="30"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="25" t="s">
+      <c r="E37" s="31"/>
+      <c r="F37" s="31"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="45"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="K37" s="23"/>
-      <c r="L37" s="42"/>
+      <c r="K37" s="31"/>
+      <c r="L37" s="39"/>
       <c r="M37" s="11" t="s">
         <v>15</v>
       </c>
@@ -6011,18 +5959,18 @@
       <c r="X37" s="14"/>
     </row>
     <row r="38" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="22"/>
-      <c r="B38" s="43"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="44"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="24"/>
-      <c r="J38" s="26"/>
-      <c r="K38" s="24"/>
-      <c r="L38" s="44"/>
+      <c r="A38" s="50"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="44"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="48"/>
+      <c r="I38" s="43"/>
+      <c r="J38" s="44"/>
+      <c r="K38" s="43"/>
+      <c r="L38" s="42"/>
       <c r="M38" s="12"/>
       <c r="N38" s="6"/>
       <c r="O38" s="6"/>
@@ -6038,6 +5986,244 @@
     </row>
   </sheetData>
   <mergeCells count="262">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="A9:A18"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="A29:A38"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="H37:H38"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="K37:K38"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="L33:L34"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="O29:O30"/>
+    <mergeCell ref="P29:P30"/>
+    <mergeCell ref="Q29:Q30"/>
+    <mergeCell ref="R29:R30"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="O23:O24"/>
+    <mergeCell ref="P23:P24"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="Q31:Q32"/>
+    <mergeCell ref="R31:R32"/>
+    <mergeCell ref="S23:S24"/>
+    <mergeCell ref="T23:T24"/>
+    <mergeCell ref="U23:U24"/>
+    <mergeCell ref="V23:V24"/>
+    <mergeCell ref="S31:S32"/>
+    <mergeCell ref="T31:T32"/>
+    <mergeCell ref="U31:U32"/>
+    <mergeCell ref="V31:V32"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="V11:V12"/>
+    <mergeCell ref="W11:W12"/>
+    <mergeCell ref="X11:X12"/>
+    <mergeCell ref="W31:W32"/>
+    <mergeCell ref="X31:X32"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="W3:W4"/>
+    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="W23:W24"/>
+    <mergeCell ref="X23:X24"/>
+    <mergeCell ref="S29:S30"/>
+    <mergeCell ref="T29:T30"/>
+    <mergeCell ref="U29:U30"/>
+    <mergeCell ref="V29:V30"/>
+    <mergeCell ref="W29:W30"/>
+    <mergeCell ref="X29:X30"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="W9:W10"/>
+    <mergeCell ref="X9:X10"/>
     <mergeCell ref="S1:X1"/>
     <mergeCell ref="M21:R21"/>
     <mergeCell ref="M1:R1"/>
@@ -6062,244 +6248,6 @@
     <mergeCell ref="S11:S12"/>
     <mergeCell ref="T11:T12"/>
     <mergeCell ref="U11:U12"/>
-    <mergeCell ref="V11:V12"/>
-    <mergeCell ref="W11:W12"/>
-    <mergeCell ref="X11:X12"/>
-    <mergeCell ref="W31:W32"/>
-    <mergeCell ref="X31:X32"/>
-    <mergeCell ref="S3:S4"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="W3:W4"/>
-    <mergeCell ref="X3:X4"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="W23:W24"/>
-    <mergeCell ref="X23:X24"/>
-    <mergeCell ref="S29:S30"/>
-    <mergeCell ref="T29:T30"/>
-    <mergeCell ref="U29:U30"/>
-    <mergeCell ref="V29:V30"/>
-    <mergeCell ref="W29:W30"/>
-    <mergeCell ref="X29:X30"/>
-    <mergeCell ref="Q31:Q32"/>
-    <mergeCell ref="R31:R32"/>
-    <mergeCell ref="S23:S24"/>
-    <mergeCell ref="T23:T24"/>
-    <mergeCell ref="U23:U24"/>
-    <mergeCell ref="V23:V24"/>
-    <mergeCell ref="S31:S32"/>
-    <mergeCell ref="T31:T32"/>
-    <mergeCell ref="U31:U32"/>
-    <mergeCell ref="V31:V32"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="O29:O30"/>
-    <mergeCell ref="P29:P30"/>
-    <mergeCell ref="Q29:Q30"/>
-    <mergeCell ref="R29:R30"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="P23:P24"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="V9:V10"/>
-    <mergeCell ref="W9:W10"/>
-    <mergeCell ref="X9:X10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="L37:L38"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="I37:I38"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="K37:K38"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="L33:L34"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="H37:H38"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="O31:O32"/>
-    <mergeCell ref="P31:P32"/>
-    <mergeCell ref="A29:A38"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="K27:K28"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="A9:A18"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>